<commit_message>
feat: land Dig camera fog overlay, map tiles, and HUD layering (v0.83.04)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/挖坟_挖坟配置表_Dig_DigGameplayConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/挖坟_挖坟配置表_Dig_DigGameplayConfig.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Work\Cursor\Gravedigger2026\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Mode2\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\CursorGame_Git\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Mode2\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255"/>
+    <workbookView windowWidth="25600" windowHeight="12080"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>玩法配置ID</t>
   </si>
@@ -135,6 +135,9 @@
     <t>Dig_02</t>
   </si>
   <si>
+    <t>Ground_02</t>
+  </si>
+  <si>
     <t>2;3</t>
   </si>
   <si>
@@ -142,6 +145,9 @@
   </si>
   <si>
     <t>Dig_03</t>
+  </si>
+  <si>
+    <t>Ground_03</t>
   </si>
   <si>
     <t>2;4</t>
@@ -1135,9 +1141,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5" outlineLevelCol="5"/>
   <cols>
-    <col min="2" max="2" width="14.25" customWidth="1"/>
+    <col min="2" max="2" width="14.2545454545455" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1225,7 +1231,7 @@
         <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C5">
         <v>50</v>
@@ -1234,18 +1240,18 @@
         <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C6">
         <v>50</v>
@@ -1254,10 +1260,10 @@
         <v>14</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>